<commit_message>
Started moving spike-in info to cbatch files.
</commit_message>
<xml_diff>
--- a/analysis/resources/PLATES_v2.0.0/CB[BATCH_ID].xlsx
+++ b/analysis/resources/PLATES_v2.0.0/CB[BATCH_ID].xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/PLATES_v2.0.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE8E6A2-17A3-8949-8522-988466857135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9425BCAE-5B57-5A4E-9E5B-ADFCEABFEAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6460" yWindow="1580" windowWidth="23220" windowHeight="14800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1240" yWindow="760" windowWidth="23420" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>

</xml_diff>